<commit_message>
feat: add external game module runtime capabilities
</commit_message>
<xml_diff>
--- a/game_config/Datas/AoiConfig.xlsx
+++ b/game_config/Datas/AoiConfig.xlsx
@@ -1,31 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\gitee\TiangZ\game_config\Datas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UGit\TiangZ\outputs\wow335-aoi-20260903\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CC75D10-C42B-4C29-9481-EB2FB52DEF57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA67B050-FCA1-403C-A038-893F9F889FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="1260" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AoiConfig" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
   <si>
     <t>##var</t>
   </si>
@@ -82,6 +77,10 @@
   </si>
   <si>
     <t>3D Demo宽视野AOI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Large World AOI</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -429,17 +428,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="39.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.53515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="39.69140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="45.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -459,7 +458,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -479,7 +478,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -499,7 +498,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -519,7 +518,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>1</v>
       </c>
@@ -536,7 +535,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>2</v>
       </c>
@@ -551,6 +550,23 @@
       </c>
       <c r="F6">
         <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7">
+        <v>15</v>
+      </c>
+      <c r="E7">
+        <v>15</v>
+      </c>
+      <c r="F7">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>